<commit_message>
Drop Evening time block — Conestoga uses Morning + Afternoon only
User's actual form has just two time blocks (Morning open-12, Afternoon
12-close). Removing the third option:

- build-template.py: heatmap is now 4 campuses x 2 time blocks (was 4x3),
  driven by TIME_BLOCK_PREFIXES list. Conditional formatting range
  derives from the list length so future changes flex.
- generate-test-data.py: drops Evening from the random distribution
  and updates the Afternoon hour range to 12-19 (since afternoon now
  spans through end of day). Regenerated test files reflect the change:
  410 people helped, 578 inquiries, all in Morning or Afternoon.
- Docs updated: volunteer-instructions, forms-build-guide,
  option-a-form-spec, shannon-reporting-notes, excel-dashboard-build-guide
  no longer mention Evening.
</commit_message>
<xml_diff>
--- a/templates/student-engagement-dashboard-starter.xlsx
+++ b/templates/student-engagement-dashboard-starter.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gabri\Documents\Project Files\Github\student-engagement\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CFAD3B4-AFF1-4C0C-8960-8F200BE9DCA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A3D97D7-6319-4134-962F-708C1E810F62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="95">
   <si>
     <t>How to use this workbook (v2 — long-format)</t>
   </si>
@@ -167,9 +167,6 @@
   </si>
   <si>
     <t>Afternoon</t>
-  </si>
-  <si>
-    <t>Evening</t>
   </si>
   <si>
     <t>Waterloo</t>
@@ -705,7 +702,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{0000000B-B30B-4A8A-9296-1D384DB80283}"/>
+              <c16:uniqueId val="{0000000B-94C8-4EDF-82BB-21F83DEFD3E1}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -719,11 +716,11 @@
         </c:dLbls>
         <c:gapWidth val="219"/>
         <c:overlap val="-27"/>
-        <c:axId val="972983744"/>
-        <c:axId val="972991904"/>
+        <c:axId val="114690992"/>
+        <c:axId val="114718352"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="972983744"/>
+        <c:axId val="114690992"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -766,7 +763,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="972991904"/>
+        <c:crossAx val="114718352"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -774,7 +771,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="972991904"/>
+        <c:axId val="114718352"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -825,7 +822,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="972983744"/>
+        <c:crossAx val="114690992"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1028,7 +1025,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{0000000B-0D59-4E75-BC65-27D4494E809F}"/>
+              <c16:uniqueId val="{0000000B-1B24-4062-8DF0-D2F210CDCEEA}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1042,11 +1039,11 @@
         </c:dLbls>
         <c:gapWidth val="219"/>
         <c:overlap val="-27"/>
-        <c:axId val="972990944"/>
-        <c:axId val="972982784"/>
+        <c:axId val="114718832"/>
+        <c:axId val="114719312"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="972990944"/>
+        <c:axId val="114718832"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1089,7 +1086,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="972982784"/>
+        <c:crossAx val="114719312"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1097,7 +1094,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="972982784"/>
+        <c:axId val="114719312"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1148,7 +1145,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="972990944"/>
+        <c:crossAx val="114718832"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1351,7 +1348,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{0000000B-8803-411D-B9B3-319CFC2A5D2C}"/>
+              <c16:uniqueId val="{0000000B-0F4A-4D42-941C-B0CCDE7BEA17}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1365,11 +1362,11 @@
         </c:dLbls>
         <c:gapWidth val="219"/>
         <c:overlap val="-27"/>
-        <c:axId val="972978944"/>
-        <c:axId val="972992864"/>
+        <c:axId val="114725072"/>
+        <c:axId val="114725552"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="972978944"/>
+        <c:axId val="114725072"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1412,7 +1409,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="972992864"/>
+        <c:crossAx val="114725552"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1420,7 +1417,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="972992864"/>
+        <c:axId val="114725552"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1471,7 +1468,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="972978944"/>
+        <c:crossAx val="114725072"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3193,7 +3190,7 @@
             <xdr:cNvPr id="2" name="slCampus">
               <a:extLst>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D600BEC0-61F6-F70E-A26D-B85C9235F9EB}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5CE9154D-7464-0BC2-15BC-2B5B2BD499AA}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -3271,7 +3268,7 @@
             <xdr:cNvPr id="3" name="slTime">
               <a:extLst>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9C95D746-F290-0B59-E45C-8E8942C676A9}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D41E4B91-F184-1A37-4DAF-031B172140A8}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -3347,7 +3344,7 @@
         <xdr:cNvPr id="4" name="chTopCategories">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C2B5FF3B-C1E9-9946-ACC0-C0E1A1EDF5E9}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FAD7C1B7-1E82-DBAB-790A-554894475908}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3383,7 +3380,7 @@
         <xdr:cNvPr id="5" name="chOutreachThemes">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D69364F0-CCEB-3CB5-5E59-87627B001B7D}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{084F433F-6154-2083-3FD3-5CAE8CAE2067}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3419,7 +3416,7 @@
         <xdr:cNvPr id="6" name="chOutreachByCampus">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6800CA24-29A9-963E-E506-F7D706396A3D}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5524B474-1756-F5DE-0EE4-EC9C644B543B}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3441,7 +3438,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Gabriel Elias Gabrie Kattan" refreshedDate="46147.820775231485" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="3" xr:uid="{487A8BB3-6719-4684-A36E-D58B084C6269}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Gabriel Elias Gabrie Kattan" refreshedDate="46147.909967245374" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="3" xr:uid="{15E29573-6556-460B-B42C-E8895C5CF0D0}">
   <cacheSource type="worksheet">
     <worksheetSource name="tblVisitor"/>
   </cacheSource>
@@ -3556,14 +3553,14 @@
   </cacheFields>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
-      <x14:pivotCacheDefinition pivotCacheId="1083663819"/>
+      <x14:pivotCacheDefinition pivotCacheId="1720447323"/>
     </ext>
   </extLst>
 </pivotCacheDefinition>
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Gabriel Elias Gabrie Kattan" refreshedDate="46147.820779166665" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="3" xr:uid="{29FDED5C-D45E-410C-A1AF-024DD98828B8}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Gabriel Elias Gabrie Kattan" refreshedDate="46147.909968981483" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="3" xr:uid="{FB1B596D-3A38-43C1-B11C-C29472C024FC}">
   <cacheSource type="worksheet">
     <worksheetSource name="tblVisitorLong"/>
   </cacheSource>
@@ -3604,7 +3601,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Gabriel Elias Gabrie Kattan" refreshedDate="46147.820788888886" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="3" xr:uid="{BCDBE610-5152-4118-B353-CCCC8F7BCE83}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Gabriel Elias Gabrie Kattan" refreshedDate="46147.909971064815" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="3" xr:uid="{2E899657-6675-4E31-801E-2DDC6905AD6D}">
   <cacheSource type="worksheet">
     <worksheetSource name="tblOutreach"/>
   </cacheSource>
@@ -3833,7 +3830,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{16C8CC98-62E0-4963-817E-18A684A81D2E}" name="ptOutreachByCampus" cacheId="17" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{445CCE66-0C77-4ADA-8D39-E361D39B3973}" name="ptOutreachByCampus" cacheId="17" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
   <location ref="J1:K3" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="9">
     <pivotField showAll="0"/>
@@ -3892,7 +3889,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{B7E51020-C0DC-4E0E-BC9C-98DFD9107402}" name="ptOutreachThemes" cacheId="17" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{8A5839FE-CDC3-41F0-872B-CBF1238A199C}" name="ptOutreachThemes" cacheId="17" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
   <location ref="G1:H3" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="9">
     <pivotField showAll="0"/>
@@ -3951,7 +3948,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{EAA0FC79-74EC-462F-8883-BC857E166A82}" name="ptTopCategories" cacheId="11" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{B2429748-13AC-47EB-A479-75BF456C5E71}" name="ptTopCategories" cacheId="11" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
   <location ref="D1:E3" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="8">
     <pivotField showAll="0"/>
@@ -4009,7 +4006,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{BC194E73-8C73-4EA3-BE42-A5387AD0CDAA}" name="ptSlicerHost" cacheId="7" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D2632FF1-CC1C-4EEA-B938-480EA2E86A63}" name="ptSlicerHost" cacheId="7" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A1:B3" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="33">
     <pivotField showAll="0"/>
@@ -4086,7 +4083,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{B3D2BBFF-1ED6-44F6-AF36-6A915727236E}" name="ptWeekly" cacheId="7" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{EC2CE0DE-279C-49DE-AE78-0B25BA0D594A}" name="ptWeekly" cacheId="7" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="B10:D15" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="33">
     <pivotField compact="0" outline="0" showAll="0"/>
@@ -4184,7 +4181,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E1519812-928F-49FB-9BB8-9A18DC4B6F78}" name="ptMonthly" cacheId="7" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3EB5CEA2-D40C-44E3-BE49-AB2DE4A7C27E}" name="ptMonthly" cacheId="7" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="B10:D15" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="33">
     <pivotField compact="0" outline="0" showAll="0"/>
@@ -4282,14 +4279,14 @@
 </file>
 
 <file path=xl/slicerCaches/slicerCache1.xml><?xml version="1.0" encoding="utf-8"?>
-<slicerCacheDefinition xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10" name="Slicer_Campus" xr10:uid="{6FFC4AAF-2EDA-4E74-8ACB-DDEBAB39CD72}" sourceName="Campus">
+<slicerCacheDefinition xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10" name="Slicer_Campus" xr10:uid="{90926E5A-871A-47DF-8A96-4B397F03F501}" sourceName="Campus">
   <pivotTables>
     <pivotTable tabId="9" name="ptSlicerHost"/>
     <pivotTable tabId="6" name="ptWeekly"/>
     <pivotTable tabId="7" name="ptMonthly"/>
   </pivotTables>
   <data>
-    <tabular pivotCacheId="1083663819">
+    <tabular pivotCacheId="1720447323">
       <items count="1">
         <i x="0" s="1"/>
       </items>
@@ -4299,14 +4296,14 @@
 </file>
 
 <file path=xl/slicerCaches/slicerCache2.xml><?xml version="1.0" encoding="utf-8"?>
-<slicerCacheDefinition xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10" name="Slicer_Time_block_this_submission_covers" xr10:uid="{77A5B991-6AC6-45AF-A5F8-03B3853F763F}" sourceName="Time block this submission covers">
+<slicerCacheDefinition xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10" name="Slicer_Time_block_this_submission_covers" xr10:uid="{BD82BD19-4ED7-486E-B6B2-D1C2096EE3F9}" sourceName="Time block this submission covers">
   <pivotTables>
     <pivotTable tabId="9" name="ptSlicerHost"/>
     <pivotTable tabId="6" name="ptWeekly"/>
     <pivotTable tabId="7" name="ptMonthly"/>
   </pivotTables>
   <data>
-    <tabular pivotCacheId="1083663819">
+    <tabular pivotCacheId="1720447323">
       <items count="1">
         <i x="0" s="1"/>
       </items>
@@ -4317,8 +4314,8 @@
 
 <file path=xl/slicers/slicer1.xml><?xml version="1.0" encoding="utf-8"?>
 <slicers xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10">
-  <slicer name="slCampus" xr10:uid="{4E123A26-8547-46FC-89A9-A1181CAB6CB7}" cache="Slicer_Campus" caption="Campus" rowHeight="241300"/>
-  <slicer name="slTime" xr10:uid="{E5DBE88E-79C5-4F2E-A7C5-78D757E966C8}" cache="Slicer_Time_block_this_submission_covers" caption="Time block" rowHeight="241300"/>
+  <slicer name="slCampus" xr10:uid="{0AFB37A0-7B1A-4099-9AD9-DAC3CFA79AF5}" cache="Slicer_Campus" caption="Campus" rowHeight="241300"/>
+  <slicer name="slTime" xr10:uid="{2CD86B23-26C0-44CA-B022-39E09C9D813E}" cache="Slicer_Time_block_this_submission_covers" caption="Time block" rowHeight="241300"/>
 </slicers>
 </file>
 
@@ -4683,7 +4680,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7BB1910-138A-4E77-94D7-C0C06EF0F329}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{536AEC31-D21E-4C2F-9BD3-AB97CD3DA31E}">
   <dimension ref="A1:K3"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
@@ -4699,51 +4696,51 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A1" s="23" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B1" t="s">
+        <v>92</v>
+      </c>
+      <c r="D1" s="23" t="s">
+        <v>89</v>
+      </c>
+      <c r="E1" t="s">
         <v>93</v>
       </c>
-      <c r="D1" s="23" t="s">
-        <v>90</v>
-      </c>
-      <c r="E1" t="s">
+      <c r="G1" s="23" t="s">
+        <v>89</v>
+      </c>
+      <c r="H1" t="s">
         <v>94</v>
       </c>
-      <c r="G1" s="23" t="s">
-        <v>90</v>
-      </c>
-      <c r="H1" t="s">
-        <v>95</v>
-      </c>
       <c r="J1" s="23" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="K1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A2" s="24" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B2" s="25">
         <v>0</v>
       </c>
       <c r="D2" s="24" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E2" s="26">
         <v>0</v>
       </c>
       <c r="G2" s="24" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H2" s="26">
         <v>0</v>
       </c>
       <c r="J2" s="24" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="K2" s="26">
         <v>0</v>
@@ -4751,25 +4748,25 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A3" s="24" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B3" s="25">
         <v>0</v>
       </c>
       <c r="D3" s="24" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E3" s="26">
         <v>0</v>
       </c>
       <c r="G3" s="24" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H3" s="26">
         <v>0</v>
       </c>
       <c r="J3" s="24" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="K3" s="26">
         <v>0</v>
@@ -5068,13 +5065,10 @@
       <c r="C8" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="D8" s="5" t="s">
-        <v>36</v>
-      </c>
     </row>
     <row r="9" spans="1:12" ht="28.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9" s="6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B9" s="7">
         <f>IFERROR(SUMIFS(tblVisitor[How many people did you help during this time block?],tblVisitor[Campus],"Waterloo",tblVisitor[Time block this submission covers],"Morning*"),0)</f>
@@ -5084,14 +5078,10 @@
         <f>IFERROR(SUMIFS(tblVisitor[How many people did you help during this time block?],tblVisitor[Campus],"Waterloo",tblVisitor[Time block this submission covers],"Afternoon*"),0)</f>
         <v>0</v>
       </c>
-      <c r="D9" s="7">
-        <f>IFERROR(SUMIFS(tblVisitor[How many people did you help during this time block?],tblVisitor[Campus],"Waterloo",tblVisitor[Time block this submission covers],"Evening*"),0)</f>
-        <v>0</v>
-      </c>
     </row>
     <row r="10" spans="1:12" ht="28.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A10" s="6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B10" s="7">
         <f>IFERROR(SUMIFS(tblVisitor[How many people did you help during this time block?],tblVisitor[Campus],"Doon",tblVisitor[Time block this submission covers],"Morning*"),0)</f>
@@ -5101,14 +5091,10 @@
         <f>IFERROR(SUMIFS(tblVisitor[How many people did you help during this time block?],tblVisitor[Campus],"Doon",tblVisitor[Time block this submission covers],"Afternoon*"),0)</f>
         <v>0</v>
       </c>
-      <c r="D10" s="7">
-        <f>IFERROR(SUMIFS(tblVisitor[How many people did you help during this time block?],tblVisitor[Campus],"Doon",tblVisitor[Time block this submission covers],"Evening*"),0)</f>
-        <v>0</v>
-      </c>
     </row>
     <row r="11" spans="1:12" ht="28.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A11" s="6" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B11" s="7">
         <f>IFERROR(SUMIFS(tblVisitor[How many people did you help during this time block?],tblVisitor[Campus],"Reuter",tblVisitor[Time block this submission covers],"Morning*"),0)</f>
@@ -5118,14 +5104,10 @@
         <f>IFERROR(SUMIFS(tblVisitor[How many people did you help during this time block?],tblVisitor[Campus],"Reuter",tblVisitor[Time block this submission covers],"Afternoon*"),0)</f>
         <v>0</v>
       </c>
-      <c r="D11" s="7">
-        <f>IFERROR(SUMIFS(tblVisitor[How many people did you help during this time block?],tblVisitor[Campus],"Reuter",tblVisitor[Time block this submission covers],"Evening*"),0)</f>
-        <v>0</v>
-      </c>
     </row>
     <row r="12" spans="1:12" ht="28.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A12" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B12" s="7">
         <f>IFERROR(SUMIFS(tblVisitor[How many people did you help during this time block?],tblVisitor[Campus],"Cambridge",tblVisitor[Time block this submission covers],"Morning*"),0)</f>
@@ -5135,14 +5117,10 @@
         <f>IFERROR(SUMIFS(tblVisitor[How many people did you help during this time block?],tblVisitor[Campus],"Cambridge",tblVisitor[Time block this submission covers],"Afternoon*"),0)</f>
         <v>0</v>
       </c>
-      <c r="D12" s="7">
-        <f>IFERROR(SUMIFS(tblVisitor[How many people did you help during this time block?],tblVisitor[Campus],"Cambridge",tblVisitor[Time block this submission covers],"Evening*"),0)</f>
-        <v>0</v>
-      </c>
     </row>
     <row r="14" spans="1:12" ht="22.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A14" s="15" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B14" s="14"/>
       <c r="C14" s="14"/>
@@ -5154,7 +5132,7 @@
     </row>
     <row r="30" spans="1:8" ht="22.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A30" s="15" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B30" s="14"/>
       <c r="C30" s="14"/>
@@ -5166,7 +5144,7 @@
     </row>
     <row r="46" spans="1:8" ht="22.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A46" s="15" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B46" s="14"/>
       <c r="C46" s="14"/>
@@ -5178,7 +5156,7 @@
     </row>
     <row r="62" spans="1:8" ht="22.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A62" s="15" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B62" s="14"/>
       <c r="C62" s="14"/>
@@ -5190,7 +5168,7 @@
     </row>
     <row r="63" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A63" s="21" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B63" s="14"/>
       <c r="C63" s="14"/>
@@ -5244,7 +5222,7 @@
     <mergeCell ref="G4:I4"/>
     <mergeCell ref="J5:L5"/>
   </mergeCells>
-  <conditionalFormatting sqref="B9:D12">
+  <conditionalFormatting sqref="B9:C12">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -5305,103 +5283,103 @@
   <sheetData>
     <row r="1" spans="1:33" ht="28.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A1" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="B1" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="C1" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="D1" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="E1" s="8" t="s">
         <v>49</v>
-      </c>
-      <c r="E1" s="8" t="s">
-        <v>50</v>
       </c>
       <c r="F1" s="8" t="s">
         <v>33</v>
       </c>
       <c r="G1" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="H1" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="H1" s="8" t="s">
+      <c r="I1" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="I1" s="8" t="s">
+      <c r="J1" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="J1" s="8" t="s">
+      <c r="K1" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="K1" s="8" t="s">
+      <c r="L1" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="L1" s="8" t="s">
+      <c r="M1" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="M1" s="8" t="s">
+      <c r="N1" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="N1" s="8" t="s">
+      <c r="O1" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="O1" s="8" t="s">
+      <c r="P1" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="P1" s="8" t="s">
+      <c r="Q1" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="Q1" s="8" t="s">
+      <c r="R1" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="R1" s="8" t="s">
+      <c r="S1" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="S1" s="8" t="s">
+      <c r="T1" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="T1" s="8" t="s">
+      <c r="U1" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="U1" s="8" t="s">
+      <c r="V1" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="V1" s="8" t="s">
+      <c r="W1" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="W1" s="8" t="s">
+      <c r="X1" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="X1" s="8" t="s">
+      <c r="Y1" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="Y1" s="8" t="s">
+      <c r="Z1" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="Z1" s="8" t="s">
+      <c r="AA1" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="AA1" s="8" t="s">
+      <c r="AB1" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="AB1" s="8" t="s">
+      <c r="AC1" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="AC1" s="8" t="s">
+      <c r="AD1" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="AD1" s="8" t="s">
+      <c r="AE1" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="AE1" s="8" t="s">
+      <c r="AF1" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="AF1" s="8" t="s">
+      <c r="AG1" s="8" t="s">
         <v>76</v>
-      </c>
-      <c r="AG1" s="8" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="2" spans="1:33" x14ac:dyDescent="0.45">
@@ -5685,31 +5663,31 @@
   <sheetData>
     <row r="1" spans="1:9" ht="28.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A1" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="B1" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="C1" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="D1" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="E1" s="8" t="s">
         <v>49</v>
-      </c>
-      <c r="E1" s="8" t="s">
-        <v>50</v>
       </c>
       <c r="F1" s="8" t="s">
         <v>33</v>
       </c>
       <c r="G1" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="H1" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="H1" s="8" t="s">
+      <c r="I1" s="8" t="s">
         <v>79</v>
-      </c>
-      <c r="I1" s="8" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.45">
@@ -5785,28 +5763,28 @@
   <sheetData>
     <row r="1" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A1" s="8" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B1" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="C1" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="D1" s="8" t="s">
         <v>49</v>
-      </c>
-      <c r="D1" s="8" t="s">
-        <v>50</v>
       </c>
       <c r="E1" s="8" t="s">
         <v>33</v>
       </c>
       <c r="F1" s="8" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G1" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="H1" s="8" t="s">
         <v>81</v>
-      </c>
-      <c r="H1" s="8" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.45">
@@ -5817,7 +5795,7 @@
         <v>45292</v>
       </c>
       <c r="G2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="H2">
         <v>0</v>
@@ -5831,7 +5809,7 @@
         <v>45458</v>
       </c>
       <c r="G3" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="H3">
         <v>0</v>
@@ -5845,7 +5823,7 @@
         <v>45657</v>
       </c>
       <c r="G4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="H4">
         <v>0</v>
@@ -5872,12 +5850,12 @@
   <sheetData>
     <row r="1" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.7">
       <c r="B1" s="11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="3" spans="2:8" ht="70.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B3" s="21" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C3" s="14"/>
       <c r="D3" s="14"/>
@@ -5924,7 +5902,7 @@
     </row>
     <row r="10" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B10" s="23" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C10" s="23" t="s">
         <v>33</v>
@@ -5932,13 +5910,13 @@
     </row>
     <row r="11" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B11" s="23" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C11" t="s">
+        <v>90</v>
+      </c>
+      <c r="D11" t="s">
         <v>91</v>
-      </c>
-      <c r="D11" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="12" spans="2:8" x14ac:dyDescent="0.45">
@@ -5976,7 +5954,7 @@
     </row>
     <row r="15" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B15" s="9" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C15" s="26">
         <v>0</v>
@@ -6006,12 +5984,12 @@
   <sheetData>
     <row r="1" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.7">
       <c r="B1" s="11" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="3" spans="2:8" ht="70.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B3" s="21" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C3" s="14"/>
       <c r="D3" s="14"/>
@@ -6058,7 +6036,7 @@
     </row>
     <row r="10" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B10" s="23" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C10" s="23" t="s">
         <v>33</v>
@@ -6066,13 +6044,13 @@
     </row>
     <row r="11" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B11" s="23" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C11" t="s">
+        <v>90</v>
+      </c>
+      <c r="D11" t="s">
         <v>91</v>
-      </c>
-      <c r="D11" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="12" spans="2:8" x14ac:dyDescent="0.45">
@@ -6110,7 +6088,7 @@
     </row>
     <row r="15" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B15" s="9" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C15" s="26">
         <v>0</v>
@@ -6137,7 +6115,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A1" s="22" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B1" s="14"/>
     </row>
@@ -6146,12 +6124,12 @@
         <v>33</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B4">
         <f>IFERROR(SUMIFS(tblVisitor[How many people did you help during this time block?],tblVisitor[Campus],"Waterloo"),0)</f>
@@ -6160,7 +6138,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B5">
         <f>IFERROR(SUMIFS(tblVisitor[How many people did you help during this time block?],tblVisitor[Campus],"Doon"),0)</f>
@@ -6169,7 +6147,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B6">
         <f>IFERROR(SUMIFS(tblVisitor[How many people did you help during this time block?],tblVisitor[Campus],"Reuter"),0)</f>
@@ -6178,7 +6156,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B7">
         <f>IFERROR(SUMIFS(tblVisitor[How many people did you help during this time block?],tblVisitor[Campus],"Cambridge"),0)</f>

</xml_diff>

<commit_message>
Use @ROWS in KPI subtext formulas to prevent #SPILL! errors
</commit_message>
<xml_diff>
--- a/templates/student-engagement-dashboard-starter.xlsx
+++ b/templates/student-engagement-dashboard-starter.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gabri\Documents\Project Files\Github\student-engagement\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A3D97D7-6319-4134-962F-708C1E810F62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B78381F-E7FD-49E6-91BB-E7DEABBCEBE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -702,7 +702,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{0000000B-94C8-4EDF-82BB-21F83DEFD3E1}"/>
+              <c16:uniqueId val="{0000000B-D9BB-46F9-A1CE-325219A356CD}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -716,11 +716,11 @@
         </c:dLbls>
         <c:gapWidth val="219"/>
         <c:overlap val="-27"/>
-        <c:axId val="114690992"/>
-        <c:axId val="114718352"/>
+        <c:axId val="1655276575"/>
+        <c:axId val="1655273215"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="114690992"/>
+        <c:axId val="1655276575"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -763,7 +763,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="114718352"/>
+        <c:crossAx val="1655273215"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -771,7 +771,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="114718352"/>
+        <c:axId val="1655273215"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -822,7 +822,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="114690992"/>
+        <c:crossAx val="1655276575"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1025,7 +1025,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{0000000B-1B24-4062-8DF0-D2F210CDCEEA}"/>
+              <c16:uniqueId val="{0000000B-AA1A-46BB-A9D0-0703B046F4B7}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1039,11 +1039,11 @@
         </c:dLbls>
         <c:gapWidth val="219"/>
         <c:overlap val="-27"/>
-        <c:axId val="114718832"/>
-        <c:axId val="114719312"/>
+        <c:axId val="1657044783"/>
+        <c:axId val="1657046223"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="114718832"/>
+        <c:axId val="1657044783"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1086,7 +1086,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="114719312"/>
+        <c:crossAx val="1657046223"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1094,7 +1094,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="114719312"/>
+        <c:axId val="1657046223"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1145,7 +1145,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="114718832"/>
+        <c:crossAx val="1657044783"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1348,7 +1348,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{0000000B-0F4A-4D42-941C-B0CCDE7BEA17}"/>
+              <c16:uniqueId val="{0000000B-CEF2-498A-A8D2-419DDDEC1456}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1362,11 +1362,11 @@
         </c:dLbls>
         <c:gapWidth val="219"/>
         <c:overlap val="-27"/>
-        <c:axId val="114725072"/>
-        <c:axId val="114725552"/>
+        <c:axId val="1689541023"/>
+        <c:axId val="1689540063"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="114725072"/>
+        <c:axId val="1689541023"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1409,7 +1409,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="114725552"/>
+        <c:crossAx val="1689540063"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1417,7 +1417,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="114725552"/>
+        <c:axId val="1689540063"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1468,7 +1468,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="114725072"/>
+        <c:crossAx val="1689541023"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3190,7 +3190,7 @@
             <xdr:cNvPr id="2" name="slCampus">
               <a:extLst>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5CE9154D-7464-0BC2-15BC-2B5B2BD499AA}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2519DC2A-3064-C4E3-FB34-BC3A949330DD}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -3268,7 +3268,7 @@
             <xdr:cNvPr id="3" name="slTime">
               <a:extLst>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D41E4B91-F184-1A37-4DAF-031B172140A8}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{75463019-B81C-22CC-B923-626402C34FD3}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -3344,7 +3344,7 @@
         <xdr:cNvPr id="4" name="chTopCategories">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FAD7C1B7-1E82-DBAB-790A-554894475908}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FF4F240B-5FC9-DC17-D8FC-679D8E5B6ECB}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3380,7 +3380,7 @@
         <xdr:cNvPr id="5" name="chOutreachThemes">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{084F433F-6154-2083-3FD3-5CAE8CAE2067}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0A1EA85E-1EE1-5068-2DB8-962EA082871C}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3416,7 +3416,7 @@
         <xdr:cNvPr id="6" name="chOutreachByCampus">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5524B474-1756-F5DE-0EE4-EC9C644B543B}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C3932D8E-4814-B889-C74D-069CCFAC7970}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3438,7 +3438,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Gabriel Elias Gabrie Kattan" refreshedDate="46147.909967245374" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="3" xr:uid="{15E29573-6556-460B-B42C-E8895C5CF0D0}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Gabriel Elias Gabrie Kattan" refreshedDate="46147.918485416667" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="3" xr:uid="{3F104E7A-8C07-4276-98A4-879A5F04A823}">
   <cacheSource type="worksheet">
     <worksheetSource name="tblVisitor"/>
   </cacheSource>
@@ -3553,14 +3553,14 @@
   </cacheFields>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
-      <x14:pivotCacheDefinition pivotCacheId="1720447323"/>
+      <x14:pivotCacheDefinition pivotCacheId="716333530"/>
     </ext>
   </extLst>
 </pivotCacheDefinition>
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Gabriel Elias Gabrie Kattan" refreshedDate="46147.909968981483" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="3" xr:uid="{FB1B596D-3A38-43C1-B11C-C29472C024FC}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Gabriel Elias Gabrie Kattan" refreshedDate="46147.918488078707" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="3" xr:uid="{9B9C7C03-C9F8-4C16-82C1-ED5751AE2227}">
   <cacheSource type="worksheet">
     <worksheetSource name="tblVisitorLong"/>
   </cacheSource>
@@ -3601,7 +3601,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Gabriel Elias Gabrie Kattan" refreshedDate="46147.909971064815" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="3" xr:uid="{2E899657-6675-4E31-801E-2DDC6905AD6D}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Gabriel Elias Gabrie Kattan" refreshedDate="46147.918489814816" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="3" xr:uid="{6D18B7C2-3AD9-4C5B-A2EC-40EA72E4E21E}">
   <cacheSource type="worksheet">
     <worksheetSource name="tblOutreach"/>
   </cacheSource>
@@ -3830,7 +3830,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{445CCE66-0C77-4ADA-8D39-E361D39B3973}" name="ptOutreachByCampus" cacheId="17" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{F60A1B92-2C6C-4A72-9732-139FFA979D59}" name="ptOutreachByCampus" cacheId="17" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
   <location ref="J1:K3" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="9">
     <pivotField showAll="0"/>
@@ -3889,7 +3889,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{8A5839FE-CDC3-41F0-872B-CBF1238A199C}" name="ptOutreachThemes" cacheId="17" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E244B785-C4B8-4F4C-BFBB-91911063FA07}" name="ptOutreachThemes" cacheId="17" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
   <location ref="G1:H3" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="9">
     <pivotField showAll="0"/>
@@ -3948,7 +3948,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{B2429748-13AC-47EB-A479-75BF456C5E71}" name="ptTopCategories" cacheId="11" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{F81A376A-57B2-4D3A-976B-E2A1FB335487}" name="ptTopCategories" cacheId="11" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
   <location ref="D1:E3" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="8">
     <pivotField showAll="0"/>
@@ -4006,7 +4006,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D2632FF1-CC1C-4EEA-B938-480EA2E86A63}" name="ptSlicerHost" cacheId="7" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D8E3A76D-E36B-4C66-B6AF-FED0A7021955}" name="ptSlicerHost" cacheId="7" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A1:B3" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="33">
     <pivotField showAll="0"/>
@@ -4083,7 +4083,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{EC2CE0DE-279C-49DE-AE78-0B25BA0D594A}" name="ptWeekly" cacheId="7" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{65A70C08-C4A3-4602-8846-13524AB14E2B}" name="ptWeekly" cacheId="7" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="B10:D15" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="33">
     <pivotField compact="0" outline="0" showAll="0"/>
@@ -4181,7 +4181,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3EB5CEA2-D40C-44E3-BE49-AB2DE4A7C27E}" name="ptMonthly" cacheId="7" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{38ECA955-0239-4850-9452-0D49E5EA8943}" name="ptMonthly" cacheId="7" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="B10:D15" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="33">
     <pivotField compact="0" outline="0" showAll="0"/>
@@ -4279,14 +4279,14 @@
 </file>
 
 <file path=xl/slicerCaches/slicerCache1.xml><?xml version="1.0" encoding="utf-8"?>
-<slicerCacheDefinition xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10" name="Slicer_Campus" xr10:uid="{90926E5A-871A-47DF-8A96-4B397F03F501}" sourceName="Campus">
+<slicerCacheDefinition xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10" name="Slicer_Campus" xr10:uid="{A8A8AF23-6B14-4997-9A14-16D1174948B2}" sourceName="Campus">
   <pivotTables>
     <pivotTable tabId="9" name="ptSlicerHost"/>
     <pivotTable tabId="6" name="ptWeekly"/>
     <pivotTable tabId="7" name="ptMonthly"/>
   </pivotTables>
   <data>
-    <tabular pivotCacheId="1720447323">
+    <tabular pivotCacheId="716333530">
       <items count="1">
         <i x="0" s="1"/>
       </items>
@@ -4296,14 +4296,14 @@
 </file>
 
 <file path=xl/slicerCaches/slicerCache2.xml><?xml version="1.0" encoding="utf-8"?>
-<slicerCacheDefinition xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10" name="Slicer_Time_block_this_submission_covers" xr10:uid="{BD82BD19-4ED7-486E-B6B2-D1C2096EE3F9}" sourceName="Time block this submission covers">
+<slicerCacheDefinition xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10" name="Slicer_Time_block_this_submission_covers" xr10:uid="{76158DB2-C97D-4CAB-82B1-30598A8C811E}" sourceName="Time block this submission covers">
   <pivotTables>
     <pivotTable tabId="9" name="ptSlicerHost"/>
     <pivotTable tabId="6" name="ptWeekly"/>
     <pivotTable tabId="7" name="ptMonthly"/>
   </pivotTables>
   <data>
-    <tabular pivotCacheId="1720447323">
+    <tabular pivotCacheId="716333530">
       <items count="1">
         <i x="0" s="1"/>
       </items>
@@ -4314,8 +4314,8 @@
 
 <file path=xl/slicers/slicer1.xml><?xml version="1.0" encoding="utf-8"?>
 <slicers xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10">
-  <slicer name="slCampus" xr10:uid="{0AFB37A0-7B1A-4099-9AD9-DAC3CFA79AF5}" cache="Slicer_Campus" caption="Campus" rowHeight="241300"/>
-  <slicer name="slTime" xr10:uid="{2CD86B23-26C0-44CA-B022-39E09C9D813E}" cache="Slicer_Time_block_this_submission_covers" caption="Time block" rowHeight="241300"/>
+  <slicer name="slCampus" xr10:uid="{49CDC992-1D9D-4589-B40A-C409BB7374BD}" cache="Slicer_Campus" caption="Campus" rowHeight="241300"/>
+  <slicer name="slTime" xr10:uid="{F4CD45CC-DCC4-4633-9C2E-C14D8F3CD2C4}" cache="Slicer_Time_block_this_submission_covers" caption="Time block" rowHeight="241300"/>
 </slicers>
 </file>
 
@@ -4680,7 +4680,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{536AEC31-D21E-4C2F-9BD3-AB97CD3DA31E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{53BCE8E1-B6A4-44F5-AFF9-2CFE7C6765B2}">
   <dimension ref="A1:K3"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
@@ -5020,7 +5020,7 @@
     </row>
     <row r="6" spans="1:12" ht="16.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="13" t="str">
-        <f>IFERROR(ROWS(tblVisitor[Id])&amp;" submissions","No data yet")</f>
+        <f>IFERROR(_xlfn.SINGLE(ROWS(tblVisitor[Id]))&amp;" submissions","No data yet")</f>
         <v>3 submissions</v>
       </c>
       <c r="B6" s="14"/>
@@ -5037,7 +5037,7 @@
       <c r="H6" s="14"/>
       <c r="I6" s="14"/>
       <c r="J6" s="13" t="str">
-        <f>IFERROR(ROWS(tblOutreach[Id])&amp;" outreach entries","")</f>
+        <f>IFERROR(_xlfn.SINGLE(ROWS(tblOutreach[Id]))&amp;" outreach entries","")</f>
         <v>3 outreach entries</v>
       </c>
       <c r="K6" s="14"/>

</xml_diff>

<commit_message>
Set MissingItemsLimit=None on all pivot caches so slicers don't show stale values
</commit_message>
<xml_diff>
--- a/templates/student-engagement-dashboard-starter.xlsx
+++ b/templates/student-engagement-dashboard-starter.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gabri\Documents\Project Files\Github\student-engagement\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B78381F-E7FD-49E6-91BB-E7DEABBCEBE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D94FEF6-9DFB-4624-854D-EC980550073C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,9 +29,9 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="7" r:id="rId10"/>
-    <pivotCache cacheId="11" r:id="rId11"/>
-    <pivotCache cacheId="17" r:id="rId12"/>
+    <pivotCache cacheId="8" r:id="rId10"/>
+    <pivotCache cacheId="13" r:id="rId11"/>
+    <pivotCache cacheId="20" r:id="rId12"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{BBE1A952-AA13-448e-AADC-164F8A28A991}">
@@ -702,7 +702,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{0000000B-D9BB-46F9-A1CE-325219A356CD}"/>
+              <c16:uniqueId val="{0000000B-AC7C-4C01-9541-BD9FA3EBBF34}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -716,11 +716,11 @@
         </c:dLbls>
         <c:gapWidth val="219"/>
         <c:overlap val="-27"/>
-        <c:axId val="1655276575"/>
-        <c:axId val="1655273215"/>
+        <c:axId val="1814496399"/>
+        <c:axId val="1814498319"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1655276575"/>
+        <c:axId val="1814496399"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -763,7 +763,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1655273215"/>
+        <c:crossAx val="1814498319"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -771,7 +771,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1655273215"/>
+        <c:axId val="1814498319"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -822,7 +822,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1655276575"/>
+        <c:crossAx val="1814496399"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1025,7 +1025,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{0000000B-AA1A-46BB-A9D0-0703B046F4B7}"/>
+              <c16:uniqueId val="{0000000B-E097-456A-A9DD-542AB29E5B2A}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1039,11 +1039,11 @@
         </c:dLbls>
         <c:gapWidth val="219"/>
         <c:overlap val="-27"/>
-        <c:axId val="1657044783"/>
-        <c:axId val="1657046223"/>
+        <c:axId val="1816751119"/>
+        <c:axId val="1816748719"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1657044783"/>
+        <c:axId val="1816751119"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1086,7 +1086,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1657046223"/>
+        <c:crossAx val="1816748719"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1094,7 +1094,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1657046223"/>
+        <c:axId val="1816748719"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1145,7 +1145,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1657044783"/>
+        <c:crossAx val="1816751119"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1348,7 +1348,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{0000000B-CEF2-498A-A8D2-419DDDEC1456}"/>
+              <c16:uniqueId val="{0000000B-E8EB-4D7F-8CF7-2C2199EC62F9}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1362,11 +1362,11 @@
         </c:dLbls>
         <c:gapWidth val="219"/>
         <c:overlap val="-27"/>
-        <c:axId val="1689541023"/>
-        <c:axId val="1689540063"/>
+        <c:axId val="1854031007"/>
+        <c:axId val="1816749679"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1689541023"/>
+        <c:axId val="1854031007"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1409,7 +1409,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1689540063"/>
+        <c:crossAx val="1816749679"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1417,7 +1417,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1689540063"/>
+        <c:axId val="1816749679"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1468,7 +1468,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1689541023"/>
+        <c:crossAx val="1854031007"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3190,7 +3190,7 @@
             <xdr:cNvPr id="2" name="slCampus">
               <a:extLst>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2519DC2A-3064-C4E3-FB34-BC3A949330DD}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E2EE4573-54C7-6B75-D50D-4DB992D5CFB2}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -3268,7 +3268,7 @@
             <xdr:cNvPr id="3" name="slTime">
               <a:extLst>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{75463019-B81C-22CC-B923-626402C34FD3}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F35D2769-93D8-575F-2BC0-632D18940492}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -3344,7 +3344,7 @@
         <xdr:cNvPr id="4" name="chTopCategories">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FF4F240B-5FC9-DC17-D8FC-679D8E5B6ECB}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6F93B42A-FC36-95F0-48AB-7AD7DDE2CBD0}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3380,7 +3380,7 @@
         <xdr:cNvPr id="5" name="chOutreachThemes">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0A1EA85E-1EE1-5068-2DB8-962EA082871C}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{80E1728B-40C2-780E-355E-A7A4647FE2C8}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3416,7 +3416,7 @@
         <xdr:cNvPr id="6" name="chOutreachByCampus">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C3932D8E-4814-B889-C74D-069CCFAC7970}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{02397C22-D70E-92FE-9E0E-DC962C88580C}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3438,7 +3438,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Gabriel Elias Gabrie Kattan" refreshedDate="46147.918485416667" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="3" xr:uid="{3F104E7A-8C07-4276-98A4-879A5F04A823}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Gabriel Elias Gabrie Kattan" refreshedDate="46147.93053287037" missingItemsLimit="0" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="3" xr:uid="{2ABCB577-52BC-4E4D-91C5-C28F5FC06EA9}">
   <cacheSource type="worksheet">
     <worksheetSource name="tblVisitor"/>
   </cacheSource>
@@ -3553,14 +3553,14 @@
   </cacheFields>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
-      <x14:pivotCacheDefinition pivotCacheId="716333530"/>
+      <x14:pivotCacheDefinition pivotCacheId="152915111"/>
     </ext>
   </extLst>
 </pivotCacheDefinition>
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Gabriel Elias Gabrie Kattan" refreshedDate="46147.918488078707" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="3" xr:uid="{9B9C7C03-C9F8-4C16-82C1-ED5751AE2227}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Gabriel Elias Gabrie Kattan" refreshedDate="46147.930535763888" missingItemsLimit="0" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="3" xr:uid="{202BFA7F-673C-4F93-9587-1BE8E001AEC9}">
   <cacheSource type="worksheet">
     <worksheetSource name="tblVisitorLong"/>
   </cacheSource>
@@ -3601,7 +3601,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Gabriel Elias Gabrie Kattan" refreshedDate="46147.918489814816" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="3" xr:uid="{6D18B7C2-3AD9-4C5B-A2EC-40EA72E4E21E}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Gabriel Elias Gabrie Kattan" refreshedDate="46147.930537499997" missingItemsLimit="0" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="3" xr:uid="{31244992-C4C3-4025-A1AA-15315E0517FE}">
   <cacheSource type="worksheet">
     <worksheetSource name="tblOutreach"/>
   </cacheSource>
@@ -3830,7 +3830,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{F60A1B92-2C6C-4A72-9732-139FFA979D59}" name="ptOutreachByCampus" cacheId="17" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{A0654080-B3C3-474D-B59C-F6ACDBD90DE0}" name="ptOutreachByCampus" cacheId="20" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
   <location ref="J1:K3" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="9">
     <pivotField showAll="0"/>
@@ -3889,7 +3889,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E244B785-C4B8-4F4C-BFBB-91911063FA07}" name="ptOutreachThemes" cacheId="17" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{CEC00D65-9352-4E08-B9EB-5200F62C285A}" name="ptOutreachThemes" cacheId="20" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
   <location ref="G1:H3" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="9">
     <pivotField showAll="0"/>
@@ -3948,7 +3948,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{F81A376A-57B2-4D3A-976B-E2A1FB335487}" name="ptTopCategories" cacheId="11" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{339DA5B3-981A-41A5-AEAE-1A188337D4F2}" name="ptTopCategories" cacheId="13" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
   <location ref="D1:E3" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="8">
     <pivotField showAll="0"/>
@@ -4006,7 +4006,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D8E3A76D-E36B-4C66-B6AF-FED0A7021955}" name="ptSlicerHost" cacheId="7" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{1FCFFBFB-17FB-4088-B5E0-33A6001E8387}" name="ptSlicerHost" cacheId="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A1:B3" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="33">
     <pivotField showAll="0"/>
@@ -4083,7 +4083,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{65A70C08-C4A3-4602-8846-13524AB14E2B}" name="ptWeekly" cacheId="7" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{5030020B-089C-4E84-ACA6-F138E1025A3A}" name="ptWeekly" cacheId="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="B10:D15" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="33">
     <pivotField compact="0" outline="0" showAll="0"/>
@@ -4181,7 +4181,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{38ECA955-0239-4850-9452-0D49E5EA8943}" name="ptMonthly" cacheId="7" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C57B576A-A4E2-45C5-9C7F-2246C8DBC8CE}" name="ptMonthly" cacheId="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="B10:D15" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="33">
     <pivotField compact="0" outline="0" showAll="0"/>
@@ -4279,14 +4279,14 @@
 </file>
 
 <file path=xl/slicerCaches/slicerCache1.xml><?xml version="1.0" encoding="utf-8"?>
-<slicerCacheDefinition xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10" name="Slicer_Campus" xr10:uid="{A8A8AF23-6B14-4997-9A14-16D1174948B2}" sourceName="Campus">
+<slicerCacheDefinition xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10" name="Slicer_Campus" xr10:uid="{A629B34F-7BFE-43E1-854A-D7077A45BA96}" sourceName="Campus">
   <pivotTables>
     <pivotTable tabId="9" name="ptSlicerHost"/>
     <pivotTable tabId="6" name="ptWeekly"/>
     <pivotTable tabId="7" name="ptMonthly"/>
   </pivotTables>
   <data>
-    <tabular pivotCacheId="716333530">
+    <tabular pivotCacheId="152915111">
       <items count="1">
         <i x="0" s="1"/>
       </items>
@@ -4296,14 +4296,14 @@
 </file>
 
 <file path=xl/slicerCaches/slicerCache2.xml><?xml version="1.0" encoding="utf-8"?>
-<slicerCacheDefinition xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10" name="Slicer_Time_block_this_submission_covers" xr10:uid="{76158DB2-C97D-4CAB-82B1-30598A8C811E}" sourceName="Time block this submission covers">
+<slicerCacheDefinition xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10" name="Slicer_Time_block_this_submission_covers" xr10:uid="{780EE2D7-5488-4ACD-8153-D6C2D761AD6A}" sourceName="Time block this submission covers">
   <pivotTables>
     <pivotTable tabId="9" name="ptSlicerHost"/>
     <pivotTable tabId="6" name="ptWeekly"/>
     <pivotTable tabId="7" name="ptMonthly"/>
   </pivotTables>
   <data>
-    <tabular pivotCacheId="716333530">
+    <tabular pivotCacheId="152915111">
       <items count="1">
         <i x="0" s="1"/>
       </items>
@@ -4314,8 +4314,8 @@
 
 <file path=xl/slicers/slicer1.xml><?xml version="1.0" encoding="utf-8"?>
 <slicers xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10">
-  <slicer name="slCampus" xr10:uid="{49CDC992-1D9D-4589-B40A-C409BB7374BD}" cache="Slicer_Campus" caption="Campus" rowHeight="241300"/>
-  <slicer name="slTime" xr10:uid="{F4CD45CC-DCC4-4633-9C2E-C14D8F3CD2C4}" cache="Slicer_Time_block_this_submission_covers" caption="Time block" rowHeight="241300"/>
+  <slicer name="slCampus" xr10:uid="{A2BD6118-9125-49ED-BE5E-8DE8BE07C2FF}" cache="Slicer_Campus" caption="Campus" rowHeight="241300"/>
+  <slicer name="slTime" xr10:uid="{C90CEBF5-B54F-4A33-85BA-F3E0EAF0C8A8}" cache="Slicer_Time_block_this_submission_covers" caption="Time block" rowHeight="241300"/>
 </slicers>
 </file>
 
@@ -4680,7 +4680,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{53BCE8E1-B6A4-44F5-AFF9-2CFE7C6765B2}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F00F2CA1-1639-44F6-ACB5-3F1549586F01}">
   <dimension ref="A1:K3"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>

</xml_diff>